<commit_message>
corrected categories.yaml yet again
</commit_message>
<xml_diff>
--- a/data/andy_ss/vocab04.xlsx
+++ b/data/andy_ss/vocab04.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david/PycharmProjects/LearnCanto_01/data/andy_ss/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{895A72DF-28B0-244B-926A-A15E66598966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43E23B4F-CBA2-4743-AC64-6418EA57528E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25600" yWindow="620" windowWidth="25600" windowHeight="28180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,6 +19,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$F$133</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>

</xml_diff>